<commit_message>
Align declaration mapping docs
</commit_message>
<xml_diff>
--- a/最新逻辑_请优先看/报关单配置关系表.xlsx
+++ b/最新逻辑_请优先看/报关单配置关系表.xlsx
@@ -602,17 +602,17 @@
       </ns0:c>
       <ns0:c r="G9" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>是</ns0:t>
+          <ns0:t>否</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H9" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>字段映射</ns0:t>
+          <ns0:t>不使用</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I9" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>备用展示/匹配字段</ns0:t>
+          <ns0:t>当前逻辑只用 QAD PN 匹配，不使用该字段</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1213,17 +1213,17 @@
       </ns0:c>
       <ns0:c r="G22" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>是</ns0:t>
+          <ns0:t>否</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H22" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>字段映射</ns0:t>
+          <ns0:t>不使用</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I22" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>备用匹配字段</ns0:t>
+          <ns0:t>当前逻辑只用 QAD PN 匹配，不使用该字段</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1794,7 +1794,7 @@
       </ns0:c>
       <ns0:c r="F1" t="inlineStr" s="1">
         <ns0:is>
-          <ns0:t>报关单PN</ns0:t>
+          <ns0:t>历史PN（不用于匹配）</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G1" t="inlineStr" s="1">
@@ -55416,7 +55416,7 @@
     <ns0:row r="6" ht="24" customHeight="1">
       <ns0:c r="A6" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>IMOS PN</ns0:t>
+          <ns0:t>历史PN/源表IMOS PN</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="B6" t="inlineStr" s="0">
@@ -55441,7 +55441,7 @@
       </ns0:c>
       <ns0:c r="F6" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>不决定合并</ns0:t>
+          <ns0:t>不参与合并，也不用于 Invoice 与 Packing 匹配</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -57307,12 +57307,12 @@
       </ns0:c>
       <ns0:c r="C5" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>优先用 QAD PN / part_no 精确匹配；必要时可用 IMOS PN 作为备用匹配</ns0:t>
+          <ns0:t>只用 QAD PN / part_no 精确匹配；不使用 IMOS PN 作为备用匹配</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D5" t="inlineStr" s="0">
         <ns0:is>
-          <ns0:t>匹配不到重量则进入异常清单</ns0:t>
+          <ns0:t>QAD PN 匹配不到重量则进入异常清单</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>

</xml_diff>

<commit_message>
Update declaration country logic and config docs
</commit_message>
<xml_diff>
--- a/最新逻辑_请优先看/报关单配置关系表.xlsx
+++ b/最新逻辑_请优先看/报关单配置关系表.xlsx
@@ -132,9 +132,9 @@
           <t>数据来源限制</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="0">
-        <is>
-          <t>应用不得从旧 报关单读取业务数据；旧报关单/空白模板只提供格式。业务数据来自 Invoice、Packing list、Daily/商品主数据和本配置表。</t>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">应用不得从旧 报关单读取业务数据；旧报关单/空白模板只提供格式。生成文件不得保留隐藏行。业务数据来自 Invoice、Packing list、Daily/商品主数据和本配置表。</t>
         </is>
       </c>
     </row>
@@ -51289,6 +51289,168 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家/地区</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vietnam</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">越南</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">英文国家名翻译</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家/地区</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Viet Nam</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">越南</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">英文国家名翻译</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家/地区</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Italy</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">意大利</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">英文国家名翻译</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家/地区</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Italia</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">意大利</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">英文国家名翻译</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家/地区</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">United States</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">美国</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">英文国家名翻译</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家/地区</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">美国</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">英文国家名翻译</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E28"/>
 </worksheet>
@@ -52095,24 +52257,24 @@
           <t>trade_country</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="0">
-        <is>
-          <t>Invoice/Packing</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="0">
-        <is>
-          <t>表头</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr" s="0">
-        <is>
-          <t>客户/地址</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr" s="0">
-        <is>
-          <t>根据值标准化推断</t>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bill to 地址块</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bill to</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">从 Bill to 地址块识别英文国家名，并翻译成中文</t>
         </is>
       </c>
       <c r="G9" t="inlineStr" s="0">
@@ -52125,9 +52287,9 @@
           <t>是</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr" s="0">
-        <is>
-          <t>CASCO Imos Italia/CONDOVE -&gt; 意大利</t>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">例如 VINFAST/Vietnam -&gt; 越南；CASCO/Italy -&gt; 意大利</t>
         </is>
       </c>
     </row>
@@ -52142,24 +52304,24 @@
           <t>destination_country</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr" s="0">
-        <is>
-          <t>Invoice/Packing</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr" s="0">
-        <is>
-          <t>表头</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr" s="0">
-        <is>
-          <t>客户/地址</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr" s="0">
-        <is>
-          <t>根据值标准化推断</t>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ship to 地址块</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ship to</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">从 Ship to 地址块识别英文国家名，并翻译成中文</t>
         </is>
       </c>
       <c r="G10" t="inlineStr" s="0">
@@ -52172,9 +52334,9 @@
           <t>是</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr" s="0">
-        <is>
-          <t>同贸易国</t>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">运抵国用于商品行最终目的国</t>
         </is>
       </c>
     </row>
@@ -52189,24 +52351,24 @@
           <t>destination_country</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr" s="0">
-        <is>
-          <t>Invoice/Packing</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr" s="0">
-        <is>
-          <t>表头</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr" s="0">
-        <is>
-          <t>客户/地址</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr" s="0">
-        <is>
-          <t>填入每个商品项</t>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ship to 地址块</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ship to</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">固定等于运抵国 G10，不允许空白</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="0">
@@ -52219,9 +52381,9 @@
           <t>是</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr" s="0">
-        <is>
-          <t>同贸易国</t>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商品每一行 M列都填运抵国</t>
         </is>
       </c>
     </row>
@@ -53597,6 +53759,50 @@
       <c r="D17" t="inlineStr">
         <is>
           <t xml:space="preserve">新增字段名优先维护字段映射表</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家字段识别</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">贸易国=Invoice Bill to 国家；运抵国=Invoice Ship to 国家；英文国家名按值标准化表翻译成中文；最终目的国=运抵国</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">如识别不到国家，进入异常提示，不从旧报关单取值</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生成格式</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生成的报关单不得保留隐藏行；模板隐藏行在输出时全部展开</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">避免客户打开文件时看不到商品行或校验行</t>
         </is>
       </c>
     </row>
@@ -53744,6 +53950,48 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v1.2</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-28</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yu/Codex</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国家字段与格式规则</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">贸易国=Bill to 国家；运抵国=Ship to 国家；最终目的国=运抵国；英文国家名翻译成中文；生成文件不保留隐藏行</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PS26002526 / VINFAST</t>
+        </is>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">对应截图红框反馈</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H2"/>
 </worksheet>

</xml_diff>

<commit_message>
Add marker template packaging support
</commit_message>
<xml_diff>
--- a/最新逻辑_请优先看/报关单配置关系表.xlsx
+++ b/最新逻辑_请优先看/报关单配置关系表.xlsx
@@ -181,6 +181,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I38"/>
   <cols>
     <col min="1" max="1" width="13.8" customWidth="1"/>
     <col min="2" max="2" width="17.2" customWidth="1"/>
@@ -372,12 +373,12 @@
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">取下方公司名称；境外收货人优先用 Ship to，公司名为空时用 Bill to</t>
+          <t>取 Bill to 下方公司名称；境外收货人优先用 Bill to，公司名为空时用 Ship to</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">样例 VINFAST TRADING AND PRODUCTION JOINT STOCK COMPANY</t>
+          <t>Bill to 公司名优先于 Ship to</t>
         </is>
       </c>
     </row>
@@ -419,12 +420,12 @@
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">优先取 Ship to 下方公司名；地址用于推断国家/目的地</t>
+          <t>取 Ship to 下方公司名作为备用；地址用于推断国家/目的地</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ship to 公司名优先于 Bill to</t>
+          <t>仅当 Bill to 公司名为空时用于境外收货人；Ship to 地址仍用于运抵国</t>
         </is>
       </c>
     </row>
@@ -51858,6 +51859,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I32"/>
   <cols>
     <col min="1" max="1" width="13.8" customWidth="1"/>
     <col min="2" max="2" width="21.8" customWidth="1"/>
@@ -52128,12 +52130,12 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ship to / Bill to</t>
+          <t>Bill to / Ship to</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">优先取 Ship to 下方公司名；没有时取 Bill to 下方公司名</t>
+          <t>优先取 Bill to 下方公司名；没有时取 Ship to 下方公司名</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="0">
@@ -52148,7 +52150,7 @@
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">样例 VINFAST TRADING AND PRODUCTION JOINT STOCK COMPANY</t>
+          <t>境外收货人按 Bill to 优先；Ship to 仅作备用</t>
         </is>
       </c>
     </row>
@@ -53381,6 +53383,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D19"/>
   <cols>
     <col min="1" max="1" width="10.0" customWidth="1"/>
     <col min="2" max="2" width="23.0" customWidth="1"/>
@@ -53709,7 +53712,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">境外收货人优先取 Ship to 下方公司名，没有时取 Bill to 下方公司名</t>
+          <t>境外收货人优先取 Bill to 下方公司名，没有时取 Ship to 下方公司名</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -53813,6 +53816,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="10.0" customWidth="1"/>
     <col min="2" max="2" width="11.5" customWidth="1"/>
@@ -53992,6 +53996,48 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yu/Codex</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>境外收货人取值优先级调整</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>境外收货人由 Ship to 优先改为 Bill to 优先；Bill to 下方公司名为空时再取 Ship to 下方公司名</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>配置表规则检查</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>同步字段映射表、报关单字段来源表和当前匹配逻辑</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H2"/>
 </worksheet>

</xml_diff>